<commit_message>
feat: datos bancarios de proveedores (SP-2123)
Permite registrar cuenta bancaria en el proveedor, importarla y mostrarla en el Excel de compras.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Backend/public/docs/proveedores-empresas-format-cr.xlsx
+++ b/Backend/public/docs/proveedores-empresas-format-cr.xlsx
@@ -1,42 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ingal\Documents\GitHub\smartpyme\Backend\public\docs\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B76112F1-60DC-477E-A5C4-F5A4B57E2F78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{9D60928E-D431-406E-B4D7-7071ACCB71C9}"/>
+    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="15">
+  <si>
+    <t>nombre_empresa</t>
+  </si>
+  <si>
+    <t>numero_registro</t>
+  </si>
   <si>
     <t>giro</t>
   </si>
@@ -47,50 +32,69 @@
     <t>direccion</t>
   </si>
   <si>
+    <t>provincia</t>
+  </si>
+  <si>
+    <t>canton</t>
+  </si>
+  <si>
+    <t>distrito</t>
+  </si>
+  <si>
     <t>telefono</t>
   </si>
   <si>
     <t>correo</t>
   </si>
   <si>
-    <t>nombre_empresa</t>
-  </si>
-  <si>
-    <t>numero_registro</t>
-  </si>
-  <si>
-    <t>provincia</t>
-  </si>
-  <si>
-    <t>distrito</t>
-  </si>
-  <si>
-    <t>canton</t>
+    <t>Banco</t>
+  </si>
+  <si>
+    <t>Tipo_cuenta</t>
+  </si>
+  <si>
+    <t>Numero_cuenta</t>
+  </si>
+  <si>
+    <t>Titular_cuenta</t>
+  </si>
+  <si>
+    <t>Forma_pago</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="10"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -115,28 +119,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -178,7 +174,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -230,7 +226,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -282,7 +278,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -291,199 +287,254 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E418D774-0BF9-4AA5-A601-75D8BF188680}">
-  <dimension ref="A1:P1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:U1"/>
+  <sheetFormatPr defaultRowHeight="14.4" defaultColWidth="8.88671875" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="15.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.6640625" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="21" customWidth="1"/>
-    <col min="5" max="5" width="16.88671875" customWidth="1"/>
-    <col min="6" max="7" width="10.88671875" customWidth="1"/>
-    <col min="8" max="9" width="12.88671875" customWidth="1"/>
-    <col min="10" max="10" width="11.109375" customWidth="1"/>
+    <col min="1" max="1" width="15.21875" customWidth="true" style="0"/>
+    <col min="2" max="2" width="13.6640625" customWidth="true" style="0"/>
+    <col min="3" max="3" width="12" customWidth="true" style="0"/>
+    <col min="4" max="4" width="21" customWidth="true" style="0"/>
+    <col min="5" max="5" width="16.88671875" customWidth="true" style="0"/>
+    <col min="6" max="6" width="10.88671875" customWidth="true" style="0"/>
+    <col min="7" max="7" width="10.88671875" customWidth="true" style="0"/>
+    <col min="8" max="8" width="12.88671875" customWidth="true" style="0"/>
+    <col min="9" max="9" width="12.88671875" customWidth="true" style="0"/>
+    <col min="10" max="10" width="11.109375" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" customHeight="1" ht="13.8" s="2" customFormat="1">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="P1" s="1"/>
+      <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
+      <c r="S1" s="2"/>
+      <c r="T1" s="2"/>
+      <c r="U1" s="2"/>
     </row>
   </sheetData>
+  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
+  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
+    <oddHeader/>
+    <oddFooter/>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <tableParts count="0"/>
 </worksheet>
 </file>
</xml_diff>